<commit_message>
0.5.45: the stringout-only Shot Type is pl##_avidref
Renamed from preVis (user): pl01_avidref, pl02_avidref, any case, pl_avidref meaning
pl01. Same behaviour: no colour correction, no delivery, no checks, QC-088 (info),
played as it is on the stringout and burned in <shotcode>_pl01_avidref. preVis01 is
now QC-010. The Shot Type workbook's row is renamed.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Shot_Types.xlsx
+++ b/docs/Shot_Types.xlsx
@@ -2760,7 +2760,7 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>preVis</t>
+          <t>pl##_avidref</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -2775,22 +2775,22 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Previs render: treated as a style frame is</t>
+          <t>Avid reference: treated as a style frame is</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>preVis01, preVis02, previs</t>
+          <t>pl01_avidref, pl02_avidref, pl_avidref</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>Its index, unused in any name</t>
+          <t>The plate number: pl02_avidref is burned in _pl02_avidref</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>A video render</t>
+          <t>A video</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
@@ -2875,7 +2875,7 @@
       </c>
       <c r="X18" s="10" t="inlineStr">
         <is>
-          <t>INCA5002_preVis01</t>
+          <t>INCA5002_pl01_avidref</t>
         </is>
       </c>
       <c r="Y18" s="10" t="inlineStr">
@@ -2911,12 +2911,12 @@
       <c r="AE18" s="10" t="inlineStr"/>
       <c r="AF18" s="10" t="inlineStr">
         <is>
-          <t>User, 2026-10-14: treated just like styleFrame</t>
+          <t>User, 2026-10-14: treated just like styleFrame; named pl##_avidref (it was preVis01 in 0.5.44)</t>
         </is>
       </c>
       <c r="AG18" s="10" t="inlineStr">
         <is>
-          <t>Assumed (OQ-86): it plays its cut, where a style frame holds one frame</t>
+          <t>Assumed (OQ-86): it plays its cut, where a style frame holds one frame. preVis01 is no longer read (QC-010)</t>
         </is>
       </c>
     </row>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>naming.ELEMENT_TYPES, AUX_NAMES, HDRI_KIND, LDRI_KIND, STYLE_FRAME_KIND, PREVIS_KIND</t>
+          <t>naming.ELEMENT_TYPES, AUX_NAMES, HDRI_KIND, LDRI_KIND, STYLE_FRAME_KIND, AVIDREF_KIND</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>naming.parse_shot_type, SHOT_TYPE_ALIASES; metacsv for HDRI, LDRI, styleFrame, preVis</t>
+          <t>naming.parse_shot_type, SHOT_TYPE_ALIASES; metacsv for HDRI, LDRI, styleFrame, pl##_avidref</t>
         </is>
       </c>
     </row>
@@ -4053,7 +4053,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>QC-010 Shot Type, QC-012 file missing, QC-013 two files, QC-014 unreadable, QC-066 no EDL event, QC-067 two possible events, QC-073 retimed in the EDL, and the AMF and CLF checks QC-075 to 079 and 082 (not on an HDRI, LDRI, styleFrame or preVis, which no check runs on). The Row QC column lists the rules that re-run after every edit.</t>
+          <t>QC-010 Shot Type, QC-012 file missing, QC-013 two files, QC-014 unreadable, QC-066 no EDL event, QC-067 two possible events, QC-073 retimed in the EDL, and the AMF and CLF checks QC-075 to 079 and 082 (not on an HDRI, LDRI, styleFrame or pl##_avidref, which no check runs on). The Row QC column lists the rules that re-run after every edit.</t>
         </is>
       </c>
     </row>
@@ -4107,7 +4107,7 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>PL01, PREVIS01 and COLORCHART all read the same. The tool writes the spelling in the Shot Type column.</t>
+          <t>PL01, PL01_AVIDREF and COLORCHART all read the same. The tool writes the spelling in the Shot Type column.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
0.5.46: the Avid reference is typed avidRef##
Ben will put avidRef## in the metadata, and the name may change again, so
the spelling lives in one constant, naming.AVIDREF_KIND, and metacsv's
pattern is built from it. avidRef01 (any case, bare avidRef is 01) is
QC-088 as before, burned in <shot>_avidRef01. pl01_avidref and preVis01
are QC-010. The Shot Type workbook's row is renamed.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Shot_Types.xlsx
+++ b/docs/Shot_Types.xlsx
@@ -2760,7 +2760,7 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>pl##_avidref</t>
+          <t>avidRef##</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -2780,12 +2780,12 @@
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>pl01_avidref, pl02_avidref, pl_avidref</t>
+          <t>avidRef01, avidRef02, avidRef</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>The plate number: pl02_avidref is burned in _pl02_avidref</t>
+          <t>The reference number: avidRef02 is burned in _avidRef02</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -2875,7 +2875,7 @@
       </c>
       <c r="X18" s="10" t="inlineStr">
         <is>
-          <t>INCA5002_pl01_avidref</t>
+          <t>INCA5002_avidRef01</t>
         </is>
       </c>
       <c r="Y18" s="10" t="inlineStr">
@@ -2911,12 +2911,12 @@
       <c r="AE18" s="10" t="inlineStr"/>
       <c r="AF18" s="10" t="inlineStr">
         <is>
-          <t>User, 2026-10-14: treated just like styleFrame; named pl##_avidref (it was preVis01 in 0.5.44)</t>
+          <t>User, 2026-10-14: treated just like styleFrame. User, 2026-10-15: Ben types it avidRef##; it may change again (preVis01 in 0.5.44, pl##_avidref in 0.5.45)</t>
         </is>
       </c>
       <c r="AG18" s="10" t="inlineStr">
         <is>
-          <t>Assumed (OQ-86): it plays its cut, where a style frame holds one frame. preVis01 is no longer read (QC-010)</t>
+          <t>Assumed (OQ-86): it plays its cut, where a style frame holds one frame. preVis01 and pl01_avidref are no longer read (QC-010)</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>naming.parse_shot_type, SHOT_TYPE_ALIASES; metacsv for HDRI, LDRI, styleFrame, pl##_avidref</t>
+          <t>naming.parse_shot_type, SHOT_TYPE_ALIASES; metacsv for HDRI, LDRI, styleFrame, avidRef##</t>
         </is>
       </c>
     </row>
@@ -4053,7 +4053,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>QC-010 Shot Type, QC-012 file missing, QC-013 two files, QC-014 unreadable, QC-066 no EDL event, QC-067 two possible events, QC-073 retimed in the EDL, and the AMF and CLF checks QC-075 to 079 and 082 (not on an HDRI, LDRI, styleFrame or pl##_avidref, which no check runs on). The Row QC column lists the rules that re-run after every edit.</t>
+          <t>QC-010 Shot Type, QC-012 file missing, QC-013 two files, QC-014 unreadable, QC-066 no EDL event, QC-067 two possible events, QC-073 retimed in the EDL, and the AMF and CLF checks QC-075 to 079 and 082 (not on an HDRI, LDRI, styleFrame or avidRef##, which no check runs on). The Row QC column lists the rules that re-run after every edit.</t>
         </is>
       </c>
     </row>
@@ -4107,7 +4107,7 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>PL01, PL01_AVIDREF and COLORCHART all read the same. The tool writes the spelling in the Shot Type column.</t>
+          <t>PL01, AVIDREF01 and COLORCHART all read the same. The tool writes the spelling in the Shot Type column.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
0.5.47: the Avid reference is delivered, never as an EXR
An avidRef## row now delivers one file (user, 2026-10-22): a movie or an
image sequence as <shot>_avidRef01_v01.mp4 over its cut at 24, the size it
is, with no colour transform (a Render has its colour baked in) and no
audio; a held JPG or PNG copied byte for byte; any other still as a JPG.
No size tag. It reads back as kind avidref and versions like the rest,
its mp4 is checked as a reference is (not QC-112), and it is left off the
tracker. The stringout is unchanged. Frame rate confirmed already 24.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Shot_Types.xlsx
+++ b/docs/Shot_Types.xlsx
@@ -89,7 +89,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -111,11 +111,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -151,6 +195,8 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -560,62 +606,62 @@
           <t>Identity</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="13" t="n"/>
+      <c r="G1" s="14" t="n"/>
       <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Colour</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
+      <c r="I1" s="13" t="n"/>
+      <c r="J1" s="13" t="n"/>
+      <c r="K1" s="14" t="n"/>
       <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="M1" s="3" t="n"/>
-      <c r="N1" s="3" t="n"/>
-      <c r="O1" s="3" t="n"/>
-      <c r="P1" s="3" t="n"/>
-      <c r="Q1" s="3" t="n"/>
-      <c r="R1" s="3" t="n"/>
-      <c r="S1" s="3" t="n"/>
-      <c r="T1" s="3" t="n"/>
-      <c r="U1" s="3" t="n"/>
+      <c r="M1" s="13" t="n"/>
+      <c r="N1" s="13" t="n"/>
+      <c r="O1" s="13" t="n"/>
+      <c r="P1" s="13" t="n"/>
+      <c r="Q1" s="13" t="n"/>
+      <c r="R1" s="13" t="n"/>
+      <c r="S1" s="13" t="n"/>
+      <c r="T1" s="13" t="n"/>
+      <c r="U1" s="14" t="n"/>
       <c r="V1" s="4" t="inlineStr">
         <is>
           <t>Stringout</t>
         </is>
       </c>
-      <c r="W1" s="4" t="n"/>
-      <c r="X1" s="4" t="n"/>
-      <c r="Y1" s="4" t="n"/>
-      <c r="Z1" s="4" t="n"/>
-      <c r="AA1" s="4" t="n"/>
+      <c r="W1" s="13" t="n"/>
+      <c r="X1" s="13" t="n"/>
+      <c r="Y1" s="13" t="n"/>
+      <c r="Z1" s="13" t="n"/>
+      <c r="AA1" s="14" t="n"/>
       <c r="AB1" s="5" t="inlineStr">
         <is>
           <t>QC</t>
         </is>
       </c>
-      <c r="AC1" s="5" t="n"/>
+      <c r="AC1" s="14" t="n"/>
       <c r="AD1" s="6" t="inlineStr">
         <is>
           <t>Spreadsheets</t>
         </is>
       </c>
-      <c r="AE1" s="6" t="n"/>
+      <c r="AE1" s="14" t="n"/>
       <c r="AF1" s="7" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="AG1" s="7" t="n"/>
+      <c r="AG1" s="14" t="n"/>
     </row>
     <row r="2" ht="45" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
@@ -2775,7 +2821,7 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Avid reference: treated as a style frame is</t>
+          <t>Avid reference: colour baked in, delivered as it is, never an EXR</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -2790,17 +2836,17 @@
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>A video</t>
+          <t>A Resolve pre-render (mp4 or mov, 'Render' in its name), an image sequence, or a still (one image file) held for some frames</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No (colour baked in)</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr">
         <is>
-          <t>No: no CC needed</t>
+          <t>No: colour baked in</t>
         </is>
       </c>
       <c r="J18" s="10" t="inlineStr">
@@ -2810,12 +2856,12 @@
       </c>
       <c r="K18" s="10" t="inlineStr">
         <is>
-          <t>No reference movies</t>
+          <t>Its own mp4, with no transform</t>
         </is>
       </c>
       <c r="L18" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes, never as an EXR</t>
         </is>
       </c>
       <c r="M18" s="10" t="inlineStr">
@@ -2850,17 +2896,17 @@
       </c>
       <c r="S18" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>A held still: a JPG or PNG under its own extension (lowercased); any other still becomes a JPG</t>
         </is>
       </c>
       <c r="T18" s="10" t="inlineStr">
         <is>
-          <t>Not delivered</t>
+          <t>A movie: the EDL's cut, at 24, the size it is. A still: its In frame</t>
         </is>
       </c>
       <c r="U18" s="10" t="inlineStr">
         <is>
-          <t>Nothing</t>
+          <t>INCA5002_avidRef01_v01.mp4 (or .jpg, .png), no size tag</t>
         </is>
       </c>
       <c r="V18" s="10" t="inlineStr">
@@ -2895,7 +2941,7 @@
       </c>
       <c r="AB18" s="10" t="inlineStr">
         <is>
-          <t>QC-088 only</t>
+          <t>QC-088 only; its mp4 is checked as a reference is (QC-110, 111, 113, 114, 115)</t>
         </is>
       </c>
       <c r="AC18" s="10" t="inlineStr">
@@ -2905,18 +2951,18 @@
       </c>
       <c r="AD18" s="10" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None: not on the sheet (user, 2026-10-22)</t>
         </is>
       </c>
       <c r="AE18" s="10" t="inlineStr"/>
       <c r="AF18" s="10" t="inlineStr">
         <is>
-          <t>User, 2026-10-14: treated just like styleFrame. User, 2026-10-15: Ben types it avidRef##; it may change again (preVis01 in 0.5.44, pl##_avidref in 0.5.45)</t>
+          <t>User, 2026-10-14: treated just like styleFrame. User, 2026-10-15: Ben types it avidRef##; it may change again (preVis01 in 0.5.44, pl##_avidref in 0.5.45). User, 2026-10-22: delivered, never an EXR</t>
         </is>
       </c>
       <c r="AG18" s="10" t="inlineStr">
         <is>
-          <t>Assumed (OQ-86): it plays its cut, where a style frame holds one frame. preVis01 and pl01_avidref are no longer read (QC-010)</t>
+          <t>Assumed (OQ-86): it plays its cut, where a style frame holds one frame; delivered ungraded with 'Render' in the name or not; its mp4 is silent; an EXR still goes to JPG with no view transform. preVis01 and pl01_avidref are no longer read (QC-010)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
0.5.48: a witness cam is named under the plate it covers
Ben types pl01_wit01 or pl02_wit01 in the Shot Type (user, 2026-10-23),
and all four deliverables and the burn-in carry both:
INCA5002_pl02_wit01_raw_4k_v01, ..._ref_HD_v01.mp4. The plate is read by
naming.witness_plate and carried as ShotIdentity.plate, so elem, stem,
every builder and the read-back follow. A bare wit01 names no plate and
is QC-010 with a message saying how to write it. The stringout lays a
witness over the plate it names only. An older batch loads with no
plate. Assumptions in OQ-87; the Shot Type workbook row is updated.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Shot_Types.xlsx
+++ b/docs/Shot_Types.xlsx
@@ -1355,12 +1355,12 @@
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>wit01</t>
+          <t>pl01_wit01, pl02_wit01 (the plate it covers, then its number; a bare wit01 is QC-010)</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>Its index: 01, 02 ... (bare means 01)</t>
+          <t>Its plate and its index: pl02_wit01 is witness 01 of pl02 (bare pl or wit means 01)</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -1435,10 +1435,10 @@
       </c>
       <c r="U7" s="10" t="inlineStr">
         <is>
-          <t>INCA5002_wit01_raw_4k_v01/INCA5002_wit01_raw_4k_v01.1001.exr
-INCA5002_wit01_raw_HD_v01/INCA5002_wit01_raw_HD_v01.1001.exr
-INCA5002_wit01_ref_4k_v01.mp4
-INCA5002_wit01_ref_HD_v01.mp4</t>
+          <t>INCA5002_pl01_wit01_raw_4k_v01/INCA5002_pl01_wit01_raw_4k_v01.1001.exr
+INCA5002_pl01_wit01_raw_HD_v01/INCA5002_pl01_wit01_raw_HD_v01.1001.exr
+INCA5002_pl01_wit01_ref_4k_v01.mp4
+INCA5002_pl01_wit01_ref_HD_v01.mp4</t>
         </is>
       </c>
       <c r="V7" s="10" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="X7" s="10" t="inlineStr">
         <is>
-          <t>INCA5002_wit01</t>
+          <t>INCA5002_pl01_wit01</t>
         </is>
       </c>
       <c r="Y7" s="10" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>Top right, quarter size</t>
+          <t>Top right, quarter size, over the plate it names (pl02_wit01 over pl02)</t>
         </is>
       </c>
       <c r="AB7" s="10" t="inlineStr">
@@ -1476,7 +1476,11 @@
           <t>QC-011, 018, 020, 021, 022, 023, 026, 027, 028, 030, 031, 032, 035, 036, 045, 046, 047, 009</t>
         </is>
       </c>
-      <c r="AC7" s="10" t="inlineStr"/>
+      <c r="AC7" s="10" t="inlineStr">
+        <is>
+          <t>The plate is read from the Shot Type (naming.witness_plate) and carried as ShotIdentity.plate</t>
+        </is>
+      </c>
       <c r="AD7" s="10" t="inlineStr">
         <is>
           <t>None</t>
@@ -1489,10 +1493,14 @@
       </c>
       <c r="AF7" s="10" t="inlineStr">
         <is>
-          <t>Shooters' spec (NAMING_SPEC, 2026-09-21)</t>
-        </is>
-      </c>
-      <c r="AG7" s="10" t="inlineStr"/>
+          <t>Shooters' spec (NAMING_SPEC, 2026-09-21); named under its plate, pl01_wit01 (user, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="AG7" s="10" t="inlineStr">
+        <is>
+          <t>The shooters' spec sheet still says INCA5002_wit01_...; it is out of date (user, 2026-10-23)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">

</xml_diff>

<commit_message>
0.5.49: meas and recon, numbered HDRIs, and the pre-render delivered
meas## and recon## are never colour corrected and are delivered as an
Avid reference is (user, 2026-10-27): a movie as <shot>_meas01_v01.mp4,
a still as itself or a JPG, never an EXR; burned in <shot>_meas01. recon
replaces re, and re01 is QC-010 saying to write recon01.

HDRIs and LDRIs are numbered by the Shot Type, HDRI01, HDRI02 (bare is
01), with no underscore: <shot>_pl01_HDRI02_v01.exr, burned in
<shot>_pl01_HDRI02. The Take no longer numbers them and QC-087 is
retired; the old HDRI_01 spelling still counts as a version. Ben's
pre-render is delivered beside the file as <shot>_pl01_HDRI02_v01.mp4,
coloured as the stringout shows it. Assumptions in OQ-88.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Shot_Types.xlsx
+++ b/docs/Shot_Types.xlsx
@@ -562,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG24"/>
+  <dimension ref="A1:AG26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Retired</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
@@ -1520,12 +1520,12 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Recon plate. Retired 2026-10-27 for recon (user: "It's now recon")</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>re01</t>
+          <t>Not any more: re01 is QC-010, saying to write recon01</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
@@ -1659,7 +1659,7 @@
       </c>
       <c r="AF8" s="10" t="inlineStr">
         <is>
-          <t>Shooters' spec (NAMING_SPEC, 2026-09-21)</t>
+          <t>Shooters' spec (NAMING_SPEC, 2026-09-21); retired for recon (user, 2026-10-27)</t>
         </is>
       </c>
       <c r="AG8" s="10" t="inlineStr"/>
@@ -2353,12 +2353,12 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>HDRI</t>
+          <t>HDRI, HDRI01, HDRI02 (any case)</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Not allowed: the number is the CSV's Take (HDRI2 is QC-010)</t>
+          <t>Its number: HDRI02 is HDRI02 (bare HDRI means 01); the Take no longer numbers it</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="K15" s="10" t="inlineStr">
         <is>
-          <t>No reference movies</t>
+          <t>Its pre-render's mp4: the HDRI's CC over linear Rec.709, as the stringout shows it</t>
         </is>
       </c>
       <c r="L15" s="10" t="inlineStr">
@@ -2428,12 +2428,13 @@
       </c>
       <c r="T15" s="10" t="inlineStr">
         <is>
-          <t>The whole file</t>
+          <t>The whole file; the pre-render's mp4 is the whole render</t>
         </is>
       </c>
       <c r="U15" s="10" t="inlineStr">
         <is>
-          <t>INCA5002_pl01_HDRI_01_v01.exr</t>
+          <t>INCA5002_pl01_HDRI01_v01.exr
+INCA5002_pl01_HDRI01_v01.mp4 (its pre-render, when there is one)</t>
         </is>
       </c>
       <c r="V15" s="10" t="inlineStr">
@@ -2448,7 +2449,7 @@
       </c>
       <c r="X15" s="10" t="inlineStr">
         <is>
-          <t>INCA5002_pl01_HDRI_01 (no Take added)</t>
+          <t>INCA5002_pl01_HDRI01 (no Take added)</t>
         </is>
       </c>
       <c r="Y15" s="10" t="inlineStr">
@@ -2468,12 +2469,12 @@
       </c>
       <c r="AB15" s="10" t="inlineStr">
         <is>
-          <t>QC-080, 083, 087, and QC-009 on an ungraded pre-render only</t>
+          <t>QC-080, 083, 086, and QC-009 on an ungraded pre-render only; its mp4 QC-110, 111, 113, 114, 115</t>
         </is>
       </c>
       <c r="AC15" s="10" t="inlineStr">
         <is>
-          <t>QC-080 (info) take as its number; QC-083 no pre-render; QC-087 blank Take</t>
+          <t>QC-080 (info) numbered by its Shot Type; QC-083 no pre-render (then no mp4)</t>
         </is>
       </c>
       <c r="AD15" s="10" t="inlineStr">
@@ -2484,10 +2485,14 @@
       <c r="AE15" s="10" t="inlineStr"/>
       <c r="AF15" s="10" t="inlineStr">
         <is>
-          <t>User, 2026-10-07; number is the take (user, 2026-10-12)</t>
-        </is>
-      </c>
-      <c r="AG15" s="10" t="inlineStr"/>
+          <t>User, 2026-10-07; numbered by the Shot Type, no underscore, the pre-render delivered as an mp4 (user, 2026-10-27)</t>
+        </is>
+      </c>
+      <c r="AG15" s="10" t="inlineStr">
+        <is>
+          <t>Assumed (OQ-88): the pre-render's mp4 is named as the EXR is, with .mp4; with no EXR (QC-086) nothing is delivered, the mp4 neither</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -2512,12 +2517,12 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>LDRI</t>
+          <t>LDRI, LDRI01, LDRI02 (any case)</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Not allowed: the number is the CSV's Take</t>
+          <t>As HDRI: LDRI02 is LDRI02, bare means 01</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -2542,7 +2547,7 @@
       </c>
       <c r="K16" s="10" t="inlineStr">
         <is>
-          <t>No reference movies</t>
+          <t>Its pre-render's mp4, as it is: never graded</t>
         </is>
       </c>
       <c r="L16" s="10" t="inlineStr">
@@ -2587,12 +2592,13 @@
       </c>
       <c r="T16" s="10" t="inlineStr">
         <is>
-          <t>The whole file</t>
+          <t>The whole file; the pre-render's mp4 is the whole render</t>
         </is>
       </c>
       <c r="U16" s="10" t="inlineStr">
         <is>
-          <t>INCA5002_pl01_LDRI_01_v01.jpg</t>
+          <t>INCA5002_pl01_LDRI01_v01.jpg
+INCA5002_pl01_LDRI01_v01.mp4 (its pre-render, when there is one)</t>
         </is>
       </c>
       <c r="V16" s="10" t="inlineStr">
@@ -2607,7 +2613,7 @@
       </c>
       <c r="X16" s="10" t="inlineStr">
         <is>
-          <t>INCA5002_pl01_LDRI_01 (no Take added)</t>
+          <t>INCA5002_pl01_LDRI01 (no Take added)</t>
         </is>
       </c>
       <c r="Y16" s="10" t="inlineStr">
@@ -2632,7 +2638,7 @@
       </c>
       <c r="AC16" s="10" t="inlineStr">
         <is>
-          <t>QC-080, 083, 086, 087</t>
+          <t>QC-080, 083, 086</t>
         </is>
       </c>
       <c r="AD16" s="10" t="inlineStr">
@@ -2643,7 +2649,7 @@
       <c r="AE16" s="10" t="inlineStr"/>
       <c r="AF16" s="10" t="inlineStr">
         <is>
-          <t>User, 2026-10-08</t>
+          <t>User, 2026-10-08; as HDRI (user, 2026-10-27)</t>
         </is>
       </c>
       <c r="AG16" s="10" t="inlineStr">
@@ -2975,89 +2981,345 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>meas##</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>Measurement: never colour corrected, delivered as it is, never an EXR</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>meas, meas01, meas02 (any case)</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Its number: meas02 is burned in _meas02 (bare means 01)</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>A movie or image sequence, or a still (one image file) held for some frames</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>No (colour baked in)</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>No: never colour corrected</t>
+        </is>
+      </c>
+      <c r="J19" s="10" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>Its own mp4, with no transform</t>
+        </is>
+      </c>
+      <c r="L19" s="10" t="inlineStr">
+        <is>
+          <t>Yes, never as an EXR</t>
+        </is>
+      </c>
+      <c r="M19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S19" s="10" t="inlineStr">
+        <is>
+          <t>A held still: a JPG or PNG under its own extension (lowercased); any other still becomes a JPG</t>
+        </is>
+      </c>
+      <c r="T19" s="10" t="inlineStr">
+        <is>
+          <t>A movie: the EDL's cut, at 24, the size it is. A still: its In frame</t>
+        </is>
+      </c>
+      <c r="U19" s="10" t="inlineStr">
+        <is>
+          <t>INCA5002_meas01_v01.mp4 (or .jpg, .png), no size tag</t>
+        </is>
+      </c>
+      <c r="V19" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W19" s="10" t="inlineStr">
+        <is>
+          <t>Plays its cut as it is, with no grade</t>
+        </is>
+      </c>
+      <c r="X19" s="10" t="inlineStr">
+        <is>
+          <t>INCA5002_meas01</t>
+        </is>
+      </c>
+      <c r="Y19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB19" s="10" t="inlineStr">
+        <is>
+          <t>QC-088 only; its mp4 is checked as a reference is (QC-110, 111, 113, 114, 115)</t>
+        </is>
+      </c>
+      <c r="AC19" s="10" t="inlineStr">
+        <is>
+          <t>QC-088 (info)</t>
+        </is>
+      </c>
+      <c r="AD19" s="10" t="inlineStr">
+        <is>
+          <t>None: no column on the sheet (assumed, OQ-88)</t>
+        </is>
+      </c>
+      <c r="AE19" s="10" t="inlineStr">
+        <is>
+          <t>measurement</t>
+        </is>
+      </c>
+      <c r="AF19" s="10" t="inlineStr">
+        <is>
+          <t>User, 2026-10-27: not colour corrected, so no EXR; a still delivered as a still, a movie as an mp4</t>
+        </is>
+      </c>
+      <c r="AG19" s="10" t="inlineStr">
+        <is>
+          <t>Assumed (OQ-88): delivered as an Avid reference is in every other respect (its cut, no handles, silent, an EXR or TIFF still becomes a JPG); not on the tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>recon##</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Recon: never colour corrected, delivered as it is, never an EXR; replaces re</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>recon, recon01, recon02 (any case)</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Its number: recon02 is burned in _recon02 (bare means 01)</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>A movie or image sequence, or a still (one image file) held for some frames</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>No (colour baked in)</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>No: never colour corrected</t>
+        </is>
+      </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="K20" s="10" t="inlineStr">
+        <is>
+          <t>Its own mp4, with no transform</t>
+        </is>
+      </c>
+      <c r="L20" s="10" t="inlineStr">
+        <is>
+          <t>Yes, never as an EXR</t>
+        </is>
+      </c>
+      <c r="M20" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N20" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O20" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P20" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q20" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R20" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S20" s="10" t="inlineStr">
+        <is>
+          <t>A held still: a JPG or PNG under its own extension (lowercased); any other still becomes a JPG</t>
+        </is>
+      </c>
+      <c r="T20" s="10" t="inlineStr">
+        <is>
+          <t>A movie: the EDL's cut, at 24, the size it is. A still: its In frame</t>
+        </is>
+      </c>
+      <c r="U20" s="10" t="inlineStr">
+        <is>
+          <t>INCA5002_recon01_v01.mp4 (or .jpg, .png), no size tag</t>
+        </is>
+      </c>
+      <c r="V20" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W20" s="10" t="inlineStr">
+        <is>
+          <t>Plays its cut as it is, with no grade</t>
+        </is>
+      </c>
+      <c r="X20" s="10" t="inlineStr">
+        <is>
+          <t>INCA5002_recon01</t>
+        </is>
+      </c>
+      <c r="Y20" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z20" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA20" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB20" s="10" t="inlineStr">
+        <is>
+          <t>QC-088 only; its mp4 is checked as a reference is (QC-110, 111, 113, 114, 115)</t>
+        </is>
+      </c>
+      <c r="AC20" s="10" t="inlineStr">
+        <is>
+          <t>QC-088 (info)</t>
+        </is>
+      </c>
+      <c r="AD20" s="10" t="inlineStr">
+        <is>
+          <t>None: no column on the sheet (assumed, OQ-88)</t>
+        </is>
+      </c>
+      <c r="AE20" s="10" t="inlineStr">
+        <is>
+          <t>recon</t>
+        </is>
+      </c>
+      <c r="AF20" s="10" t="inlineStr">
+        <is>
+          <t>User, 2026-10-27: not colour corrected, so no EXR; a still delivered as a still, a movie as an mp4</t>
+        </is>
+      </c>
+      <c r="AG20" s="10" t="inlineStr">
+        <is>
+          <t>Assumed (OQ-88): delivered as an Avid reference is in every other respect (its cut, no handles, silent, an EXR or TIFF still becomes a JPG); not on the tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>New types: fill in a row before it is built</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr"/>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="inlineStr"/>
-      <c r="D20" s="12" t="inlineStr"/>
-      <c r="E20" s="12" t="inlineStr"/>
-      <c r="F20" s="12" t="inlineStr"/>
-      <c r="G20" s="12" t="inlineStr"/>
-      <c r="H20" s="12" t="inlineStr"/>
-      <c r="I20" s="12" t="inlineStr"/>
-      <c r="J20" s="12" t="inlineStr"/>
-      <c r="K20" s="12" t="inlineStr"/>
-      <c r="L20" s="12" t="inlineStr"/>
-      <c r="M20" s="12" t="inlineStr"/>
-      <c r="N20" s="12" t="inlineStr"/>
-      <c r="O20" s="12" t="inlineStr"/>
-      <c r="P20" s="12" t="inlineStr"/>
-      <c r="Q20" s="12" t="inlineStr"/>
-      <c r="R20" s="12" t="inlineStr"/>
-      <c r="S20" s="12" t="inlineStr"/>
-      <c r="T20" s="12" t="inlineStr"/>
-      <c r="U20" s="12" t="inlineStr"/>
-      <c r="V20" s="12" t="inlineStr"/>
-      <c r="W20" s="12" t="inlineStr"/>
-      <c r="X20" s="12" t="inlineStr"/>
-      <c r="Y20" s="12" t="inlineStr"/>
-      <c r="Z20" s="12" t="inlineStr"/>
-      <c r="AA20" s="12" t="inlineStr"/>
-      <c r="AB20" s="12" t="inlineStr"/>
-      <c r="AC20" s="12" t="inlineStr"/>
-      <c r="AD20" s="12" t="inlineStr"/>
-      <c r="AE20" s="12" t="inlineStr"/>
-      <c r="AF20" s="12" t="inlineStr"/>
-      <c r="AG20" s="12" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr"/>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr"/>
-      <c r="D21" s="12" t="inlineStr"/>
-      <c r="E21" s="12" t="inlineStr"/>
-      <c r="F21" s="12" t="inlineStr"/>
-      <c r="G21" s="12" t="inlineStr"/>
-      <c r="H21" s="12" t="inlineStr"/>
-      <c r="I21" s="12" t="inlineStr"/>
-      <c r="J21" s="12" t="inlineStr"/>
-      <c r="K21" s="12" t="inlineStr"/>
-      <c r="L21" s="12" t="inlineStr"/>
-      <c r="M21" s="12" t="inlineStr"/>
-      <c r="N21" s="12" t="inlineStr"/>
-      <c r="O21" s="12" t="inlineStr"/>
-      <c r="P21" s="12" t="inlineStr"/>
-      <c r="Q21" s="12" t="inlineStr"/>
-      <c r="R21" s="12" t="inlineStr"/>
-      <c r="S21" s="12" t="inlineStr"/>
-      <c r="T21" s="12" t="inlineStr"/>
-      <c r="U21" s="12" t="inlineStr"/>
-      <c r="V21" s="12" t="inlineStr"/>
-      <c r="W21" s="12" t="inlineStr"/>
-      <c r="X21" s="12" t="inlineStr"/>
-      <c r="Y21" s="12" t="inlineStr"/>
-      <c r="Z21" s="12" t="inlineStr"/>
-      <c r="AA21" s="12" t="inlineStr"/>
-      <c r="AB21" s="12" t="inlineStr"/>
-      <c r="AC21" s="12" t="inlineStr"/>
-      <c r="AD21" s="12" t="inlineStr"/>
-      <c r="AE21" s="12" t="inlineStr"/>
-      <c r="AF21" s="12" t="inlineStr"/>
-      <c r="AG21" s="12" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr"/>
@@ -3176,6 +3438,84 @@
       <c r="AF24" s="12" t="inlineStr"/>
       <c r="AG24" s="12" t="inlineStr"/>
     </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr"/>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr"/>
+      <c r="D25" s="12" t="inlineStr"/>
+      <c r="E25" s="12" t="inlineStr"/>
+      <c r="F25" s="12" t="inlineStr"/>
+      <c r="G25" s="12" t="inlineStr"/>
+      <c r="H25" s="12" t="inlineStr"/>
+      <c r="I25" s="12" t="inlineStr"/>
+      <c r="J25" s="12" t="inlineStr"/>
+      <c r="K25" s="12" t="inlineStr"/>
+      <c r="L25" s="12" t="inlineStr"/>
+      <c r="M25" s="12" t="inlineStr"/>
+      <c r="N25" s="12" t="inlineStr"/>
+      <c r="O25" s="12" t="inlineStr"/>
+      <c r="P25" s="12" t="inlineStr"/>
+      <c r="Q25" s="12" t="inlineStr"/>
+      <c r="R25" s="12" t="inlineStr"/>
+      <c r="S25" s="12" t="inlineStr"/>
+      <c r="T25" s="12" t="inlineStr"/>
+      <c r="U25" s="12" t="inlineStr"/>
+      <c r="V25" s="12" t="inlineStr"/>
+      <c r="W25" s="12" t="inlineStr"/>
+      <c r="X25" s="12" t="inlineStr"/>
+      <c r="Y25" s="12" t="inlineStr"/>
+      <c r="Z25" s="12" t="inlineStr"/>
+      <c r="AA25" s="12" t="inlineStr"/>
+      <c r="AB25" s="12" t="inlineStr"/>
+      <c r="AC25" s="12" t="inlineStr"/>
+      <c r="AD25" s="12" t="inlineStr"/>
+      <c r="AE25" s="12" t="inlineStr"/>
+      <c r="AF25" s="12" t="inlineStr"/>
+      <c r="AG25" s="12" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr"/>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr"/>
+      <c r="D26" s="12" t="inlineStr"/>
+      <c r="E26" s="12" t="inlineStr"/>
+      <c r="F26" s="12" t="inlineStr"/>
+      <c r="G26" s="12" t="inlineStr"/>
+      <c r="H26" s="12" t="inlineStr"/>
+      <c r="I26" s="12" t="inlineStr"/>
+      <c r="J26" s="12" t="inlineStr"/>
+      <c r="K26" s="12" t="inlineStr"/>
+      <c r="L26" s="12" t="inlineStr"/>
+      <c r="M26" s="12" t="inlineStr"/>
+      <c r="N26" s="12" t="inlineStr"/>
+      <c r="O26" s="12" t="inlineStr"/>
+      <c r="P26" s="12" t="inlineStr"/>
+      <c r="Q26" s="12" t="inlineStr"/>
+      <c r="R26" s="12" t="inlineStr"/>
+      <c r="S26" s="12" t="inlineStr"/>
+      <c r="T26" s="12" t="inlineStr"/>
+      <c r="U26" s="12" t="inlineStr"/>
+      <c r="V26" s="12" t="inlineStr"/>
+      <c r="W26" s="12" t="inlineStr"/>
+      <c r="X26" s="12" t="inlineStr"/>
+      <c r="Y26" s="12" t="inlineStr"/>
+      <c r="Z26" s="12" t="inlineStr"/>
+      <c r="AA26" s="12" t="inlineStr"/>
+      <c r="AB26" s="12" t="inlineStr"/>
+      <c r="AC26" s="12" t="inlineStr"/>
+      <c r="AD26" s="12" t="inlineStr"/>
+      <c r="AE26" s="12" t="inlineStr"/>
+      <c r="AF26" s="12" t="inlineStr"/>
+      <c r="AG26" s="12" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="V1:AA1"/>
@@ -3185,14 +3525,14 @@
     <mergeCell ref="A3:AG3"/>
     <mergeCell ref="AF1:AG1"/>
     <mergeCell ref="AD1:AE1"/>
-    <mergeCell ref="A19:AG19"/>
+    <mergeCell ref="A21:AG21"/>
     <mergeCell ref="H1:K1"/>
     <mergeCell ref="L1:U1"/>
     <mergeCell ref="A14:AG14"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="B3:B74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Built,Proposed"</formula1>
+      <formula1>"Built,Proposed,Retired"</formula1>
     </dataValidation>
     <dataValidation sqref="C3:C74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Element,Reference still,Special"</formula1>

</xml_diff>

<commit_message>
0.5.52: US spelling, color everywhere
Every "colour" in code, UI, the Fix-it report, QC messages, spreadsheets
and docs is now "color" (a US company; the British spelling confused
people). COLOUR_SESSION_EXPORT.md is COLOR_SESSION_EXPORT.md. The H.264
field names colour_primaries and colour_description_present_flag stay
as the standard spells them. Adds docs/Shot_Types.docx.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Shot_Types.xlsx
+++ b/docs/Shot_Types.xlsx
@@ -614,7 +614,7 @@
       <c r="G1" s="14" t="n"/>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Colour</t>
+          <t>Color</t>
         </is>
       </c>
       <c r="I1" s="13" t="n"/>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Colour chart</t>
+          <t>Color chart</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="AE10" s="10" t="inlineStr">
         <is>
-          <t>colour chart</t>
+          <t>color chart</t>
         </is>
       </c>
       <c r="AF10" s="10" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Avid reference: colour baked in, delivered as it is, never an EXR</t>
+          <t>Avid reference: color baked in, delivered as it is, never an EXR</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -2855,12 +2855,12 @@
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>No (colour baked in)</t>
+          <t>No (color baked in)</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr">
         <is>
-          <t>No: colour baked in</t>
+          <t>No: color baked in</t>
         </is>
       </c>
       <c r="J18" s="10" t="inlineStr">
@@ -2998,7 +2998,7 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>Measurement: never colour corrected, delivered as it is, never an EXR</t>
+          <t>Measurement: never color corrected, delivered as it is, never an EXR</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
@@ -3018,12 +3018,12 @@
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>No (colour baked in)</t>
+          <t>No (color baked in)</t>
         </is>
       </c>
       <c r="I19" s="10" t="inlineStr">
         <is>
-          <t>No: never colour corrected</t>
+          <t>No: never color corrected</t>
         </is>
       </c>
       <c r="J19" s="10" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="AF19" s="10" t="inlineStr">
         <is>
-          <t>User, 2026-10-27: not colour corrected, so no EXR; a still delivered as a still, a movie as an mp4</t>
+          <t>User, 2026-10-27: not color corrected, so no EXR; a still delivered as a still, a movie as an mp4</t>
         </is>
       </c>
       <c r="AG19" s="10" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>Recon: never colour corrected, delivered as it is, never an EXR; replaces re</t>
+          <t>Recon: never color corrected, delivered as it is, never an EXR; replaces re</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
@@ -3185,12 +3185,12 @@
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>No (colour baked in)</t>
+          <t>No (color baked in)</t>
         </is>
       </c>
       <c r="I20" s="10" t="inlineStr">
         <is>
-          <t>No: never colour corrected</t>
+          <t>No: never color corrected</t>
         </is>
       </c>
       <c r="J20" s="10" t="inlineStr">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="AF20" s="10" t="inlineStr">
         <is>
-          <t>User, 2026-10-27: not colour corrected, so no EXR; a still delivered as a still, a movie as an mp4</t>
+          <t>User, 2026-10-27: not color corrected, so no EXR; a still delivered as a still, a movie as an mp4</t>
         </is>
       </c>
       <c r="AG20" s="10" t="inlineStr">
@@ -3732,7 +3732,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Colour</t>
+          <t>Color</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -3754,7 +3754,7 @@
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Colour</t>
+          <t>Color</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
@@ -3776,7 +3776,7 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Colour</t>
+          <t>Color</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
@@ -3798,7 +3798,7 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Colour</t>
+          <t>Color</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
@@ -4394,7 +4394,7 @@
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Colour</t>
+          <t>Color</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">

</xml_diff>

<commit_message>
0.5.53: turnover150, the stringout builds and an HDRI delivers its mp4
- The stringout read a cut by the file's own timecode alone; C2098.MP4's
  is six seconds off Resolve's Start TC, so it asked for frames before
  the file began. Scan and stringout now share scan.cut_in_file.
- An HDRI or LDRI delivers only its pre-render as an mp4. The EXR or
  image is Ben's to deliver by hand and is never looked for; QC-086 is
  retired. The tracker's HDRI column names the mp4.
- A shot's colorChart02 is no longer folded into its colorChart01.
- A stringout segment whose file decodes a frame or two short holds its
  last frame instead of failing the stringout.

Verified on Windows against the turnover150 folder on G: 10,787 frames.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Shot_Types.xlsx
+++ b/docs/Shot_Types.xlsx
@@ -2363,7 +2363,7 @@
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>An EXR; Ben's pre-render of its timeline event beside it (&lt;EXR name&gt; Render 1.mov)</t>
+          <t>Ben's pre-render of its timeline event, a movie (e.g. INCA3001_pl01_HDRI01_Render.mov). The EXR is not looked for: Ben delivers it by hand</t>
         </is>
       </c>
       <c r="H15" s="10" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="L15" s="10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes: the pre-render's mp4 only</t>
         </is>
       </c>
       <c r="M15" s="10" t="inlineStr">
@@ -2423,18 +2423,17 @@
       </c>
       <c r="S15" s="10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No (until 2026-10-30)</t>
         </is>
       </c>
       <c r="T15" s="10" t="inlineStr">
         <is>
-          <t>The whole file; the pre-render's mp4 is the whole render</t>
+          <t>The whole render</t>
         </is>
       </c>
       <c r="U15" s="10" t="inlineStr">
         <is>
-          <t>INCA5002_pl01_HDRI01_v01.exr
-INCA5002_pl01_HDRI01_v01.mp4 (its pre-render, when there is one)</t>
+          <t>INCA5002_pl01_HDRI01_v01.mp4 (its pre-render). The EXR is Ben's to deliver by hand</t>
         </is>
       </c>
       <c r="V15" s="10" t="inlineStr">
@@ -2444,7 +2443,7 @@
       </c>
       <c r="W15" s="10" t="inlineStr">
         <is>
-          <t>Ben's pre-render, read as linear Rec.709, with the HDRI's CC; the EXR held if there is no pre-render</t>
+          <t>Ben's pre-render, read as linear Rec.709, with the HDRI's CC; black if the pre-render is missing</t>
         </is>
       </c>
       <c r="X15" s="10" t="inlineStr">
@@ -2469,28 +2468,28 @@
       </c>
       <c r="AB15" s="10" t="inlineStr">
         <is>
-          <t>QC-080, 083, 086, and QC-009 on an ungraded pre-render only; its mp4 QC-110, 111, 113, 114, 115</t>
+          <t>QC-080, 083, and QC-009 on an ungraded pre-render only; its mp4 QC-110, 111, 113, 114, 115</t>
         </is>
       </c>
       <c r="AC15" s="10" t="inlineStr">
         <is>
-          <t>QC-080 (info) numbered by its Shot Type; QC-083 no pre-render (then no mp4)</t>
+          <t>QC-080 (info) numbered by its Shot Type; QC-083 no pre-render (then black on the stringout, and no mp4)</t>
         </is>
       </c>
       <c r="AD15" s="10" t="inlineStr">
         <is>
-          <t>HDRI (the delivered name)</t>
+          <t>HDRI (the pre-render's mp4, user 2026-10-30; the copied EXR before)</t>
         </is>
       </c>
       <c r="AE15" s="10" t="inlineStr"/>
       <c r="AF15" s="10" t="inlineStr">
         <is>
-          <t>User, 2026-10-07; numbered by the Shot Type, no underscore, the pre-render delivered as an mp4 (user, 2026-10-27)</t>
+          <t>User, 2026-10-07; numbered by the Shot Type, no underscore, the pre-render delivered as an mp4 (user, 2026-10-27); the EXR delivered by Ben by hand, only the pre-render's mp4 by the tool (user, 2026-10-30)</t>
         </is>
       </c>
       <c r="AG15" s="10" t="inlineStr">
         <is>
-          <t>Assumed (OQ-88): the pre-render's mp4 is named as the EXR is, with .mp4; with no EXR (QC-086) nothing is delivered, the mp4 neither</t>
+          <t>Assumed (OQ-88): the pre-render's mp4 is named as the EXR would be, with .mp4</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2526,7 @@
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>A .jpg, .jpeg or .png; its pre-render beside it (&lt;image name&gt; Render 1.mov)</t>
+          <t>Ben's pre-render of its timeline event, a movie (e.g. INCA3001_pl01_LDRI01_Render.mov). The JPG or PNG is not looked for: Ben delivers it by hand</t>
         </is>
       </c>
       <c r="H16" s="10" t="inlineStr">
@@ -2552,7 +2551,7 @@
       </c>
       <c r="L16" s="10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes: the pre-render's mp4 only</t>
         </is>
       </c>
       <c r="M16" s="10" t="inlineStr">
@@ -2587,18 +2586,17 @@
       </c>
       <c r="S16" s="10" t="inlineStr">
         <is>
-          <t>Yes, under its own extension (lowercased)</t>
+          <t>No (until 2026-10-30)</t>
         </is>
       </c>
       <c r="T16" s="10" t="inlineStr">
         <is>
-          <t>The whole file; the pre-render's mp4 is the whole render</t>
+          <t>The whole render</t>
         </is>
       </c>
       <c r="U16" s="10" t="inlineStr">
         <is>
-          <t>INCA5002_pl01_LDRI01_v01.jpg
-INCA5002_pl01_LDRI01_v01.mp4 (its pre-render, when there is one)</t>
+          <t>INCA5002_pl01_LDRI01_v01.mp4 (its pre-render). The JPG or PNG is Ben's to deliver by hand</t>
         </is>
       </c>
       <c r="V16" s="10" t="inlineStr">
@@ -2608,7 +2606,7 @@
       </c>
       <c r="W16" s="10" t="inlineStr">
         <is>
-          <t>Its pre-render, or the image held, as it is: never graded</t>
+          <t>Its pre-render, as it is: never graded; black if the pre-render is missing</t>
         </is>
       </c>
       <c r="X16" s="10" t="inlineStr">
@@ -2638,7 +2636,7 @@
       </c>
       <c r="AC16" s="10" t="inlineStr">
         <is>
-          <t>QC-080, 083, 086</t>
+          <t>QC-080 (info) numbered by its Shot Type; QC-083 no pre-render (then black on the stringout, and no mp4)</t>
         </is>
       </c>
       <c r="AD16" s="10" t="inlineStr">
@@ -2649,7 +2647,7 @@
       <c r="AE16" s="10" t="inlineStr"/>
       <c r="AF16" s="10" t="inlineStr">
         <is>
-          <t>User, 2026-10-08; as HDRI (user, 2026-10-27)</t>
+          <t>User, 2026-10-08; as HDRI (user, 2026-10-27); the JPG or PNG delivered by Ben by hand, only the pre-render's mp4 by the tool (user, 2026-10-30)</t>
         </is>
       </c>
       <c r="AG16" s="10" t="inlineStr">

</xml_diff>